<commit_message>
Tests implementation and corrections on plots
</commit_message>
<xml_diff>
--- a/examples/Imputation/Imputed_data_Example_loaded.xlsx
+++ b/examples/Imputation/Imputed_data_Example_loaded.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,86 +417,86 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Small</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Big</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>2 legs</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>4 legs</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Hair</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Hooves</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Mane</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Feather</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Hunt</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Fly</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Swin</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Dove</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.043597</v>
+        <v>0.998074</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.002148</v>
+        <v>0.010932</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.106686</v>
+        <v>-0.0007470000000000001</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -542,7 +530,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Hen</t>
         </is>
@@ -588,7 +576,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Duck</t>
         </is>
@@ -634,7 +622,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Goose</t>
         </is>
@@ -680,7 +668,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Owl</t>
         </is>
@@ -726,7 +714,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Hawk</t>
         </is>
@@ -772,7 +760,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Eagle</t>
         </is>
@@ -818,7 +806,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Fox</t>
         </is>
@@ -864,7 +852,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Dog</t>
         </is>
@@ -910,7 +898,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Wolf</t>
         </is>
@@ -956,7 +944,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Cat</t>
         </is>
@@ -1002,7 +990,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Tiger</t>
         </is>
@@ -1048,7 +1036,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Lion</t>
         </is>
@@ -1094,7 +1082,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Horse</t>
         </is>
@@ -1140,7 +1128,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Zebra</t>
         </is>
@@ -1186,7 +1174,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Cow</t>
         </is>
@@ -1232,7 +1220,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Monkey</t>
         </is>
@@ -1278,7 +1266,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Gorilla</t>
         </is>

</xml_diff>